<commit_message>
remove Spike signalProperty which is not implemented, add StableTime signalProperty which will be implemented in the next iteration
</commit_message>
<xml_diff>
--- a/infrastructure/knowledgebase/SystemData.xlsx
+++ b/infrastructure/knowledgebase/SystemData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\user1\sense\use-case-template\infrastructure\knowledgebase\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1DCFDD2-506C-4909-B590-18496EBD7201}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C053CD42-5709-4A81-8DDC-C814A3154197}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" tabRatio="608" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30612" yWindow="-108" windowWidth="30936" windowHeight="16776" tabRatio="608" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PlatformTypes" sheetId="1" r:id="rId1"/>
@@ -35,9 +35,6 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
   </extLst>
 </workbook>
@@ -210,7 +207,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="71">
   <si>
     <t>PlatformType</t>
   </si>
@@ -347,24 +344,6 @@
     <t>WithinBounds</t>
   </si>
   <si>
-    <t>Spike</t>
-  </si>
-  <si>
-    <t>amplitude1</t>
-  </si>
-  <si>
-    <t>amplitude2</t>
-  </si>
-  <si>
-    <t>slope1</t>
-  </si>
-  <si>
-    <t>slope2</t>
-  </si>
-  <si>
-    <t>width</t>
-  </si>
-  <si>
     <t>RiseTime</t>
   </si>
   <si>
@@ -426,6 +405,21 @@
   </si>
   <si>
     <t>ExampleStateType2</t>
+  </si>
+  <si>
+    <t>StableTime</t>
+  </si>
+  <si>
+    <t>maximum_delta</t>
+  </si>
+  <si>
+    <t>stable_time</t>
+  </si>
+  <si>
+    <t>CustomDefinition</t>
+  </si>
+  <si>
+    <t>implemented_in</t>
   </si>
 </sst>
 </file>
@@ -551,7 +545,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -573,16 +567,17 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Explanatory Text" xfId="1" builtinId="53"/>
@@ -670,9 +665,7 @@
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="Schreiberhuber, Katrin" id="{CE6926BB-C9BE-8A48-9527-C0157D9F0173}" userId="S::katrin.schreiberhuber@wu.ac.at::a8bbfc8c-fdf4-4b40-89d7-e571648d1de5" providerId="AD"/>
-</personList>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -848,14 +841,6 @@
 </a:theme>
 </file>
 
-<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
-<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="B1" dT="2024-08-05T14:54:41.70" personId="{CE6926BB-C9BE-8A48-9527-C0157D9F0173}" id="{09D8B89D-83C7-0A4D-A20A-A968FD3B7817}">
-    <text>Added as there was no connetion between eventTypes and sensors yet.</text>
-  </threadedComment>
-</ThreadedComments>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
@@ -878,7 +863,7 @@
     </row>
     <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -917,7 +902,7 @@
     </row>
     <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -985,10 +970,10 @@
     </row>
     <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="B2" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -3049,10 +3034,10 @@
     </row>
     <row r="2" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C2" t="b">
         <v>1</v>
@@ -3061,10 +3046,10 @@
     </row>
     <row r="3" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C3" t="b">
         <v>0</v>
@@ -3246,82 +3231,82 @@
         <v>17</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="F1" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="G1" s="14" t="s">
+      <c r="G1" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="K1" s="14"/>
+      <c r="L1" s="14"/>
+      <c r="M1" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="N1" s="14"/>
+      <c r="O1" s="14"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A2" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="K1" s="15"/>
-      <c r="L1" s="15"/>
-      <c r="M1" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="N1" s="15"/>
-      <c r="O1" s="15"/>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A2" s="16" t="s">
-        <v>64</v>
-      </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
       <c r="G2" s="11" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="H2" s="10" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="I2" s="10" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="J2" s="11" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="K2" s="10" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="L2" s="10" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="M2" s="11" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="N2" s="10" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="O2" s="10" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="B3" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="C3" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="D3" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="E3" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="F3" t="s">
         <v>30</v>
@@ -3329,14 +3314,12 @@
       <c r="G3" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="H3" s="13" t="s">
-        <v>65</v>
+      <c r="H3" t="s">
+        <v>59</v>
       </c>
       <c r="I3">
         <v>1</v>
       </c>
-      <c r="K3" s="13"/>
-      <c r="N3" s="13"/>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" s="4"/>
@@ -3372,29 +3355,29 @@
           </x14:formula1>
           <xm:sqref>E3:E1048576</xm:sqref>
         </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{3CF3A043-EA1C-4F42-937C-8B04B72FFA8D}">
+          <x14:formula1>
+            <xm:f>PlatformTypes!$A:$A</xm:f>
+          </x14:formula1>
+          <xm:sqref>D2:D1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" xr:uid="{7F5B68FC-7714-4D02-B319-4ACA1D309FCB}">
+          <x14:formula1>
+            <xm:f>IF(H3="SensorValue",SensorTypes!$A:$A,SensorTypes!$Z:$Z)</xm:f>
+          </x14:formula1>
+          <xm:sqref>O3:O1048576 I3:I1048576 L3:L1048576</xm:sqref>
+        </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{4A86B01A-D006-4896-87A4-6C2FD7644D5A}">
           <x14:formula1>
             <xm:f>SignalProperties!$A:$A</xm:f>
           </x14:formula1>
           <xm:sqref>F2:F1048576</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{3CF3A043-EA1C-4F42-937C-8B04B72FFA8D}">
-          <x14:formula1>
-            <xm:f>PlatformTypes!$A:$A</xm:f>
-          </x14:formula1>
-          <xm:sqref>D2:D1048576</xm:sqref>
-        </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{69C42B8B-2E42-4221-A6F7-F81194B80C62}">
           <x14:formula1>
             <xm:f>_xlfn.XLOOKUP($F3,SignalProperties!$A:$A,SignalProperties!$B:$K)</xm:f>
           </x14:formula1>
-          <xm:sqref>M3:M1048576 G3:G1048576 J3:J1048576</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" xr:uid="{7F5B68FC-7714-4D02-B319-4ACA1D309FCB}">
-          <x14:formula1>
-            <xm:f>IF(H3="SensorValue",SensorTypes!$A:$A,SensorTypes!$Z:$Z)</xm:f>
-          </x14:formula1>
-          <xm:sqref>O3:O1048576 I3:I1048576 L3:L1048576</xm:sqref>
+          <xm:sqref>M3:M1048576 J3:J1048576 G3:G1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -3404,7 +3387,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5824542-7FEF-412D-B84A-5B5499A18F79}">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.21875" customWidth="1"/>
@@ -3518,36 +3501,35 @@
       <c r="C6" t="s">
         <v>47</v>
       </c>
-      <c r="D6" t="s">
-        <v>48</v>
-      </c>
-      <c r="E6" t="s">
-        <v>49</v>
-      </c>
-      <c r="F6" t="s">
-        <v>50</v>
-      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B7" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="C7" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>54</v>
-      </c>
-      <c r="B8" t="s">
-        <v>52</v>
-      </c>
-      <c r="C8" t="s">
-        <v>55</v>
+      <c r="A8" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -3556,6 +3538,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100DE058F8930E0E241B4560415FE1909FD" ma:contentTypeVersion="13" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="c6bffe89e109856986e4a153dc9c9910">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e9ad02b1-1808-4f55-81c1-02da346030c9" xmlns:ns3="c4d4e922-8223-4f42-92be-35e8d7f6a6aa" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a3655badd60cf411d5bfbcddb7e8975c" ns2:_="" ns3:_="">
     <xsd:import namespace="e9ad02b1-1808-4f55-81c1-02da346030c9"/>
@@ -3762,16 +3753,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9021D77D-0171-444A-8359-A9F86F12F6AA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4E49F44B-A41E-465B-AAE6-BCCE8904B251}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3788,12 +3778,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9021D77D-0171-444A-8359-A9F86F12F6AA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>